<commit_message>
Finished list r resistant report for VN
</commit_message>
<xml_diff>
--- a/api/templates/list_r_resistant_test/en.xlsx
+++ b/api/templates/list_r_resistant_test/en.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-18.04\home\nsabaj\Repositories\aspect\api\templates\list_r_resistant_test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63830BD1-F67A-4555-8EA8-330098453DE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC053FE6-9950-4376-BD5B-07798301E2DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{0E5D046B-46E4-4AC6-B2A8-F60000E7545A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0E5D046B-46E4-4AC6-B2A8-F60000E7545A}"/>
   </bookViews>
   <sheets>
     <sheet name="List-R resistant test" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="33">
   <si>
     <t>LIST OF RIFAMPICIN RESISTANCE TESTS DETECTED BY XPERT</t>
   </si>
@@ -84,9 +84,6 @@
     <t>Total R-Resistance Tests:</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t xml:space="preserve">Date      month        year   </t>
   </si>
   <si>
@@ -117,9 +114,6 @@
     <t>&lt;Table&gt;</t>
   </si>
   <si>
-    <t>#</t>
-  </si>
-  <si>
     <t>Tel phone:</t>
   </si>
   <si>
@@ -132,17 +126,32 @@
     <t>&lt;total&gt;</t>
   </si>
   <si>
-    <t>Date Range:</t>
-  </si>
-  <si>
     <t>&lt;fill&gt;</t>
+  </si>
+  <si>
+    <t>&lt;#&gt;</t>
+  </si>
+  <si>
+    <t>&lt;UserEmail&gt;</t>
+  </si>
+  <si>
+    <t>&lt;UserMobilePhone&gt;</t>
+  </si>
+  <si>
+    <t>&lt;UserFullName&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Dates&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Sites&gt;</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -192,12 +201,6 @@
       <family val="1"/>
     </font>
     <font>
-      <sz val="14"/>
-      <color indexed="8"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -263,13 +266,6 @@
       <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -320,9 +316,9 @@
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyProtection="1">
@@ -334,9 +330,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="1" applyFont="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
       <protection locked="0"/>
@@ -349,38 +342,30 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="14" fontId="11" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="14" fontId="10" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="14" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyProtection="1">
@@ -390,20 +375,8 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="14" fontId="8" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
@@ -411,60 +384,64 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="14" fontId="10" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="15" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="11" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="16" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="17" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -783,28 +760,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{482BE919-B2BE-45CF-B921-4E468D2D3773}">
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.5" customWidth="1"/>
-    <col min="3" max="3" width="12.5" customWidth="1"/>
-    <col min="7" max="7" width="11" style="36"/>
+    <col min="2" max="2" width="19.625" customWidth="1"/>
+    <col min="3" max="3" width="8.125" customWidth="1"/>
+    <col min="7" max="7" width="11" style="21"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="1"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
     </row>
     <row r="2" spans="1:9" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A2" s="29"/>
+      <c r="A2" s="29" t="s">
+        <v>31</v>
+      </c>
       <c r="B2" s="29"/>
       <c r="C2" s="29"/>
       <c r="D2" s="29"/>
@@ -814,200 +794,200 @@
       <c r="H2" s="1"/>
     </row>
     <row r="3" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A3" s="31" t="s">
+      <c r="A3" s="26" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="26"/>
+      <c r="C3" s="33" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3" s="33"/>
+      <c r="E3" s="33"/>
+      <c r="F3" s="33"/>
+      <c r="G3" s="33"/>
+      <c r="H3" s="36"/>
+      <c r="I3" s="3"/>
+    </row>
+    <row r="4" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A4" s="37" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="37"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="34" t="s">
+        <v>29</v>
+      </c>
+      <c r="G4" s="34"/>
+      <c r="H4" s="34"/>
+      <c r="I4" s="3"/>
+    </row>
+    <row r="5" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" s="33" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" s="33"/>
+      <c r="E5" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="F5" s="35" t="s">
         <v>28</v>
       </c>
-      <c r="B3" s="31"/>
-      <c r="C3" s="31"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="35"/>
-      <c r="I3" s="3"/>
-    </row>
-    <row r="4" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A4" s="32" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="32"/>
-      <c r="C4" s="32"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="35"/>
-      <c r="H4" s="1"/>
-    </row>
-    <row r="5" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="33" t="s">
-        <v>2</v>
-      </c>
-      <c r="B5" s="33"/>
-      <c r="C5" s="33"/>
+      <c r="G5" s="35"/>
+      <c r="H5" s="35"/>
+      <c r="I5" s="3"/>
     </row>
     <row r="6" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A6" s="33" t="s">
+      <c r="A6" s="25"/>
+      <c r="B6" s="25"/>
+      <c r="C6" s="25"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="17"/>
+      <c r="I6" s="3"/>
+    </row>
+    <row r="8" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="19"/>
+      <c r="F8" s="19"/>
+      <c r="G8" s="22"/>
+      <c r="H8" s="1"/>
+    </row>
+    <row r="9" spans="1:9" ht="73.5" x14ac:dyDescent="0.2">
+      <c r="A9" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="G9" s="23" t="s">
+        <v>9</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="30" x14ac:dyDescent="0.2">
+      <c r="A10" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G10" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="H10" s="11" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="32" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="32"/>
+      <c r="C12" s="32"/>
+      <c r="D12" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="33"/>
-      <c r="C6" s="33"/>
-    </row>
-    <row r="7" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="33" t="s">
-        <v>24</v>
-      </c>
-      <c r="B7" s="33"/>
-      <c r="C7" s="33"/>
-      <c r="D7" s="21"/>
-      <c r="E7" s="21"/>
-      <c r="F7" s="21"/>
-      <c r="G7" s="37"/>
-      <c r="H7" s="21"/>
-    </row>
-    <row r="8" spans="1:9" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="33" t="s">
-        <v>26</v>
-      </c>
-      <c r="B8" s="33"/>
-      <c r="C8" s="33"/>
-      <c r="D8" s="13"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="22"/>
-      <c r="H8" s="23"/>
-    </row>
-    <row r="9" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="10" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="25"/>
-      <c r="E10" s="25"/>
-      <c r="F10" s="25"/>
-      <c r="G10" s="38"/>
-      <c r="H10" s="1"/>
-    </row>
-    <row r="11" spans="1:9" ht="73.5" x14ac:dyDescent="0.2">
-      <c r="A11" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="E11" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="F11" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="G11" s="39" t="s">
-        <v>9</v>
-      </c>
-      <c r="H11" s="8" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="30" x14ac:dyDescent="0.2">
-      <c r="A12" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="C12" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="D12" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="E12" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="F12" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="G12" s="34" t="s">
-        <v>21</v>
-      </c>
-      <c r="H12" s="12" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="30" t="s">
-        <v>11</v>
-      </c>
-      <c r="B14" s="30"/>
-      <c r="C14" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="D14" s="5" t="s">
+      <c r="E12" s="12"/>
+      <c r="F12" s="12"/>
+      <c r="G12" s="13"/>
+    </row>
+    <row r="13" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="15"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="E14" s="15"/>
-      <c r="F14" s="15"/>
-      <c r="G14" s="16"/>
-    </row>
-    <row r="15" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="18"/>
-      <c r="B15" s="18"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="18"/>
-      <c r="F15" s="24" t="s">
+      <c r="G13" s="24"/>
+      <c r="H13" s="4"/>
+    </row>
+    <row r="14" spans="1:9" ht="16.5" x14ac:dyDescent="0.2">
+      <c r="A14" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="G15" s="40"/>
-      <c r="H15" s="4"/>
-    </row>
-    <row r="16" spans="1:9" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A16" s="27" t="s">
+      <c r="B14" s="31"/>
+      <c r="C14" s="16"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="27"/>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="20" t="s">
+      <c r="F14" s="31"/>
+      <c r="G14" s="31"/>
+      <c r="H14" s="2"/>
+    </row>
+    <row r="15" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A15" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="G16" s="41"/>
-      <c r="H16" s="2"/>
-    </row>
-    <row r="17" spans="1:8" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A17" s="26" t="s">
+      <c r="B15" s="28"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="28" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="26"/>
-      <c r="C17" s="18"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="18"/>
-      <c r="F17" s="26" t="s">
-        <v>17</v>
-      </c>
-      <c r="G17" s="26"/>
+      <c r="F15" s="28"/>
+      <c r="G15" s="28"/>
+      <c r="H15" s="2"/>
+    </row>
+    <row r="17" spans="8:8" x14ac:dyDescent="0.2">
       <c r="H17" s="2"/>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="H19" s="2"/>
-    </row>
   </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A1:G1"/>
+  <mergeCells count="13">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A15:B15"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="A8:C8"/>
     <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="E14:G14"/>
+    <mergeCell ref="E15:G15"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="F4:H4"/>
+    <mergeCell ref="F5:H5"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C3:G3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Added state and notes tags to VN reports
</commit_message>
<xml_diff>
--- a/api/templates/list_r_resistant_test/en.xlsx
+++ b/api/templates/list_r_resistant_test/en.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-18.04\home\nsabaj\Repositories\aspect\api\templates\list_r_resistant_test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC053FE6-9950-4376-BD5B-07798301E2DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2756DCE4-5463-45A5-8CDD-EA111F6D4EA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0E5D046B-46E4-4AC6-B2A8-F60000E7545A}"/>
+    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{0E5D046B-46E4-4AC6-B2A8-F60000E7545A}"/>
   </bookViews>
   <sheets>
     <sheet name="List-R resistant test" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="35">
   <si>
     <t>LIST OF RIFAMPICIN RESISTANCE TESTS DETECTED BY XPERT</t>
   </si>
@@ -145,6 +145,12 @@
   </si>
   <si>
     <t>&lt;Sites&gt;</t>
+  </si>
+  <si>
+    <t>&lt;notes&gt;</t>
+  </si>
+  <si>
+    <t>&lt;States&gt;</t>
   </si>
 </sst>
 </file>
@@ -409,6 +415,7 @@
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -421,27 +428,26 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -770,27 +776,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
     </row>
     <row r="2" spans="1:9" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A2" s="29" t="s">
+      <c r="A2" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
       <c r="H2" s="1"/>
     </row>
     <row r="3" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
@@ -798,49 +804,51 @@
         <v>1</v>
       </c>
       <c r="B3" s="26"/>
-      <c r="C3" s="33" t="s">
+      <c r="C3" s="35" t="s">
         <v>32</v>
       </c>
-      <c r="D3" s="33"/>
-      <c r="E3" s="33"/>
-      <c r="F3" s="33"/>
-      <c r="G3" s="33"/>
-      <c r="H3" s="36"/>
+      <c r="D3" s="35"/>
+      <c r="E3" s="35"/>
+      <c r="F3" s="35"/>
+      <c r="G3" s="35"/>
+      <c r="H3" s="27"/>
       <c r="I3" s="3"/>
     </row>
     <row r="4" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A4" s="37" t="s">
+      <c r="A4" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="37"/>
-      <c r="C4" s="30"/>
-      <c r="D4" s="30"/>
+      <c r="B4" s="36"/>
+      <c r="C4" s="37" t="s">
+        <v>34</v>
+      </c>
+      <c r="D4" s="37"/>
       <c r="E4" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="F4" s="34" t="s">
+      <c r="F4" s="33" t="s">
         <v>29</v>
       </c>
-      <c r="G4" s="34"/>
-      <c r="H4" s="34"/>
+      <c r="G4" s="33"/>
+      <c r="H4" s="33"/>
       <c r="I4" s="3"/>
     </row>
     <row r="5" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C5" s="33" t="s">
+      <c r="C5" s="35" t="s">
         <v>30</v>
       </c>
-      <c r="D5" s="33"/>
+      <c r="D5" s="35"/>
       <c r="E5" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="F5" s="35" t="s">
+      <c r="F5" s="34" t="s">
         <v>28</v>
       </c>
-      <c r="G5" s="35"/>
-      <c r="H5" s="35"/>
+      <c r="G5" s="34"/>
+      <c r="H5" s="34"/>
       <c r="I5" s="3"/>
     </row>
     <row r="6" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
@@ -914,7 +922,7 @@
         <v>20</v>
       </c>
       <c r="H10" s="11" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -957,17 +965,17 @@
       <c r="H14" s="2"/>
     </row>
     <row r="15" spans="1:9" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A15" s="28" t="s">
+      <c r="A15" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="28"/>
+      <c r="B15" s="29"/>
       <c r="C15" s="15"/>
       <c r="D15" s="15"/>
-      <c r="E15" s="28" t="s">
+      <c r="E15" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="F15" s="28"/>
-      <c r="G15" s="28"/>
+      <c r="F15" s="29"/>
+      <c r="G15" s="29"/>
       <c r="H15" s="2"/>
     </row>
     <row r="17" spans="8:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Added target group to the List R Resistant report for VN
</commit_message>
<xml_diff>
--- a/api/templates/list_r_resistant_test/en.xlsx
+++ b/api/templates/list_r_resistant_test/en.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-18.04\home\nsabaj\Repositories\aspect\api\templates\list_r_resistant_test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2756DCE4-5463-45A5-8CDD-EA111F6D4EA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{768F8E6A-7BEF-43F4-BEE6-BE1F08000957}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{0E5D046B-46E4-4AC6-B2A8-F60000E7545A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0E5D046B-46E4-4AC6-B2A8-F60000E7545A}"/>
   </bookViews>
   <sheets>
     <sheet name="List-R resistant test" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t>LIST OF RIFAMPICIN RESISTANCE TESTS DETECTED BY XPERT</t>
   </si>
@@ -151,6 +151,9 @@
   </si>
   <si>
     <t>&lt;States&gt;</t>
+  </si>
+  <si>
+    <t>&lt;targetGroup&gt;</t>
   </si>
 </sst>
 </file>
@@ -913,7 +916,7 @@
         <v>19</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="F10" s="9" t="s">
         <v>26</v>

</xml_diff>